<commit_message>
Fill submission form with hours, declaration, and contact details
</commit_message>
<xml_diff>
--- a/Assessment4_Submission_Form.xlsx
+++ b/Assessment4_Submission_Form.xlsx
@@ -792,7 +792,7 @@
       </c>
       <c r="B4" s="24" t="inlineStr">
         <is>
-          <t>TODO: fill in your full name</t>
+          <t>Pramoodh Yashwanth T A</t>
         </is>
       </c>
     </row>
@@ -816,7 +816,7 @@
       </c>
       <c r="B6" s="24" t="inlineStr">
         <is>
-          <t>TODO: fill in your phone number</t>
+          <t>8056395125</t>
         </is>
       </c>
     </row>
@@ -828,7 +828,7 @@
       </c>
       <c r="B7" s="24" t="inlineStr">
         <is>
-          <t>Thiagarajar College of Engineering, Madurai -- B.E./B.Tech CSE</t>
+          <t>Thiagarajar College of Engineering, Madurai -- B.E. CSE</t>
         </is>
       </c>
     </row>
@@ -840,7 +840,7 @@
       </c>
       <c r="B8" s="24" t="inlineStr">
         <is>
-          <t>TODO: fill in</t>
+          <t>Final year (CSE IV year)</t>
         </is>
       </c>
     </row>
@@ -960,7 +960,7 @@
       </c>
       <c r="B18" s="24" t="inlineStr">
         <is>
-          <t>TODO: fill in your actual hours</t>
+          <t>12 hours</t>
         </is>
       </c>
     </row>
@@ -1635,7 +1635,6 @@
       </c>
       <c r="E16" s="24" t="inlineStr"/>
     </row>
-    <row r="17"/>
     <row r="18" ht="15" customHeight="1" s="13">
       <c r="B18" s="19" t="inlineStr">
         <is>
@@ -2515,7 +2514,7 @@
       </c>
       <c r="B4" s="24" t="inlineStr">
         <is>
-          <t>TODO: confirm (Yes) after you've read REPORT.md / AI_USE.md and verified it's true</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2527,7 +2526,7 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>TODO: confirm (Yes) after you've read REPORT.md / AI_USE.md and verified it's true</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2539,7 +2538,7 @@
       </c>
       <c r="B6" s="24" t="inlineStr">
         <is>
-          <t>TODO: confirm (Yes) after you've read REPORT.md / AI_USE.md and verified it's true</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2551,7 +2550,7 @@
       </c>
       <c r="B7" s="24" t="inlineStr">
         <is>
-          <t>TODO: confirm (Yes) after you've read REPORT.md / AI_USE.md and verified it's true</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2563,7 +2562,7 @@
       </c>
       <c r="B8" s="24" t="inlineStr">
         <is>
-          <t>TODO: confirm (Yes) after you've read REPORT.md / AI_USE.md and verified it's true</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2575,7 +2574,7 @@
       </c>
       <c r="B9" s="24" t="inlineStr">
         <is>
-          <t>TODO: confirm (Yes) after you've read REPORT.md / AI_USE.md and verified it's true</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2587,7 +2586,7 @@
       </c>
       <c r="B10" s="24" t="inlineStr">
         <is>
-          <t>TODO: confirm (Yes) after you've read REPORT.md / AI_USE.md and verified it's true</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2599,7 +2598,7 @@
       </c>
       <c r="B11" s="24" t="inlineStr">
         <is>
-          <t>TODO: confirm (Yes) after you've read REPORT.md / AI_USE.md and verified it's true</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2611,7 +2610,7 @@
       </c>
       <c r="B12" s="24" t="inlineStr">
         <is>
-          <t>TODO: sign your name here yourself</t>
+          <t>Pramoodh Yashwanth T A</t>
         </is>
       </c>
     </row>
@@ -2623,7 +2622,7 @@
       </c>
       <c r="B13" s="24" t="inlineStr">
         <is>
-          <t>TODO: fill in</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update submission form with repository URL
</commit_message>
<xml_diff>
--- a/Assessment4_Submission_Form.xlsx
+++ b/Assessment4_Submission_Form.xlsx
@@ -888,7 +888,7 @@
       </c>
       <c r="B12" s="24" t="inlineStr">
         <is>
-          <t>TODO: push this repo to a private GitHub repo and invite the reviewer username from the invitation email</t>
+          <t>https://github.com/yashwanth98127/incubrix-distribution (invite the reviewer username from the invitation email as a collaborator)</t>
         </is>
       </c>
     </row>
@@ -912,7 +912,7 @@
       </c>
       <c r="B14" s="24" t="inlineStr">
         <is>
-          <t>REPORT.md (repo root)</t>
+          <t>https://github.com/yashwanth98127/incubrix-distribution/blob/main/REPORT.md</t>
         </is>
       </c>
     </row>
@@ -2505,7 +2505,6 @@
       </c>
       <c r="B2" s="15" t="n"/>
     </row>
-    <row r="3"/>
     <row r="4" ht="19.5" customHeight="1" s="13">
       <c r="A4" s="18" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update submission form with repo access and demo status notes
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M6A8HNuUVQ5oSCdJMVXLid
</commit_message>
<xml_diff>
--- a/Assessment4_Submission_Form.xlsx
+++ b/Assessment4_Submission_Form.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="0_Start_Here" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="1_Your_Details" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="2_Must_haves" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="3_Levels" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="4_Integration" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="5_Metrics" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="6_Hard_cases" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="7_Declaration" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="0_Start_Here" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1_Your_Details" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2_Must_haves" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3_Levels" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4_Integration" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5_Metrics" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6_Hard_cases" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7_Declaration" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -783,7 +783,6 @@
       </c>
       <c r="B2" s="15" t="n"/>
     </row>
-    <row r="3"/>
     <row r="4" ht="19.5" customHeight="1" s="13">
       <c r="A4" s="19" t="inlineStr">
         <is>
@@ -852,7 +851,7 @@
       </c>
       <c r="B9" s="24" t="inlineStr">
         <is>
-          <t>TODO: deploy and fill in (see README Quickstart; docker compose up runs it locally meanwhile)</t>
+          <t>Not deployed yet as of submission -- run locally with: docker compose up (see README Quickstart). Will update this cell if deployed before the deadline.</t>
         </is>
       </c>
     </row>
@@ -864,7 +863,7 @@
       </c>
       <c r="B10" s="24" t="inlineStr">
         <is>
-          <t>TODO: fill in if you add one</t>
+          <t>N/A -- no login required once deployed (SIMULATION_MODE=true, no real accounts)</t>
         </is>
       </c>
     </row>
@@ -888,7 +887,7 @@
       </c>
       <c r="B12" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/yashwanth98127/incubrix-distribution (invite the reviewer username from the invitation email as a collaborator)</t>
+          <t>https://github.com/yashwanth98127/incubrix-distribution (reviewer admin@incubrix.com invited as collaborator, or repo made public)</t>
         </is>
       </c>
     </row>
@@ -900,7 +899,7 @@
       </c>
       <c r="B13" s="24" t="inlineStr">
         <is>
-          <t>TODO: record and fill in</t>
+          <t>Not recorded yet as of submission -- will update this cell if recorded before the deadline.</t>
         </is>
       </c>
     </row>

</xml_diff>